<commit_message>
BA docs: remove em dashes
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/handoff/BA-ADMIN.xlsx
+++ b/handoff/BA-ADMIN.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="612">
   <si>
-    <t>Tenderfy Super Admin — Business Analysis</t>
+    <t>Tenderfy Super Admin Business Analysis</t>
   </si>
   <si>
     <t>Initial BA documentation for the admin side of the tender-kit pipeline</t>
@@ -36,7 +36,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1 — draft for review</t>
+    <t>0.1 draft for review</t>
   </si>
   <si>
     <t>Date</t>
@@ -72,7 +72,7 @@
     <t>Evidence base</t>
   </si>
   <si>
-    <t>Derived from the working prototype at daandydoan.github.io/tenderfy-admin and decisions logged in the repo. NOT yet validated with an onboarding operator — see OQ-1.</t>
+    <t>Derived from the working prototype at daandydoan.github.io/tenderfy-admin and decisions logged in the repo. NOT yet validated with an onboarding operator. See OQ-1.</t>
   </si>
   <si>
     <t/>
@@ -87,7 +87,7 @@
     <t>Amber rows</t>
   </si>
   <si>
-    <t>Marked BLOCKING — a decision is needed before that item can be built.</t>
+    <t>Marked BLOCKING. A decision is needed before that item can be built.</t>
   </si>
   <si>
     <t>Priority column</t>
@@ -324,7 +324,7 @@
     <t>Staff roles, privacy/security pages, support content</t>
   </si>
   <si>
-    <t>—</t>
+    <t>-</t>
   </si>
   <si>
     <t>Client-side editor</t>
@@ -378,7 +378,7 @@
     <t>Needs from this work</t>
   </si>
   <si>
-    <t>Tom — founder</t>
+    <t>Tom (founder)</t>
   </si>
   <si>
     <t>Does admin-built onboarding scale; commercial model</t>
@@ -390,7 +390,7 @@
     <t>OQ-1 answered; a model defensible to prospects</t>
   </si>
   <si>
-    <t>Shivam — tech lead</t>
+    <t>Shivam (tech lead)</t>
   </si>
   <si>
     <t>Feasibility, shared component library, effort</t>
@@ -399,7 +399,7 @@
     <t>Unambiguous data model and invariants (tab 9)</t>
   </si>
   <si>
-    <t>Daniel — BA / dev / UI-UX</t>
+    <t>Daniel (BA / dev / UI-UX)</t>
   </si>
   <si>
     <t>Owns prototype and specification</t>
@@ -438,7 +438,7 @@
     <t>High (external)</t>
   </si>
   <si>
-    <t>Brand sign-off; permissions — client-side</t>
+    <t>Brand sign-off; permissions (client-side)</t>
   </si>
   <si>
     <t>Client estimator</t>
@@ -450,13 +450,13 @@
     <t>Medium (external)</t>
   </si>
   <si>
-    <t>A template that is already right — client-side</t>
+    <t>A template that is already right (client-side)</t>
   </si>
   <si>
     <t>ADMIN ROLES</t>
   </si>
   <si>
-    <t>As modelled in settings.html — see OQ-4 on whether the matrix is final</t>
+    <t>As modelled in settings.html: see OQ-4 on whether the matrix is final</t>
   </si>
   <si>
     <t>Super Admin</t>
@@ -543,7 +543,7 @@
     <t>Admin hours per client; lead time to first fillable template</t>
   </si>
   <si>
-    <t>UNKNOWN — OQ-1</t>
+    <t>UNKNOWN, see OQ-1</t>
   </si>
   <si>
     <t>The number that decides whether admin-built scales</t>
@@ -603,7 +603,7 @@
     <t>Brand</t>
   </si>
   <si>
-    <t>A versioned record of the client's visual tokens — logo, colours by role, heading/body fonts, type scale — each value tagged with its evidence</t>
+    <t>A versioned record of the client's visual tokens (logo, colours by role, heading/body fonts, type scale), each value tagged with its evidence</t>
   </si>
   <si>
     <t>The client's styleguide, proven</t>
@@ -657,7 +657,7 @@
     <t>Repeat row</t>
   </si>
   <si>
-    <t>A block row marked "one per item" — rendered once per instance at fill time</t>
+    <t>A block row marked "one per item", rendered once per instance at fill time</t>
   </si>
   <si>
     <t>One per item</t>
@@ -684,10 +684,10 @@
     <t>CONTAINMENT</t>
   </si>
   <si>
-    <t>Tender template ⊃ Documents ⊃ Blocks ⊃ Elements. Brand is not in that chain — the renderer applies it across all of it at output.</t>
-  </si>
-  <si>
-    <t>5. To-be process — the admin onboarding pipeline</t>
+    <t>Tender template ⊃ Documents ⊃ Blocks ⊃ Elements. Brand is not in that chain; the renderer applies it across all of it at output.</t>
+  </si>
+  <si>
+    <t>5. To-be process, the admin onboarding pipeline</t>
   </si>
   <si>
     <t>Nine stages from signed client to issued tender. The last row records the as-is process being replaced.</t>
@@ -834,7 +834,7 @@
     <t>6. Functional requirements</t>
   </si>
   <si>
-    <t>Feature level, for estimation — not build-ready user stories. Priority is PROPOSED by the author; confirm in review.</t>
+    <t>Feature level, for estimation, not build-ready user stories. Priority is PROPOSED by the author; confirm in review.</t>
   </si>
   <si>
     <t>Module</t>
@@ -927,7 +927,7 @@
     <t>Keep a change log of brand edits</t>
   </si>
   <si>
-    <t>See OQ-3 — log vs versions</t>
+    <t>See OQ-3, log vs versions</t>
   </si>
   <si>
     <t>FR-M3-5</t>
@@ -978,7 +978,7 @@
     <t>FR-M4-5</t>
   </si>
   <si>
-    <t>Mark a row as a repeat row (down or across) — "one per item"</t>
+    <t>Mark a row as a repeat row (down or across), "one per item"</t>
   </si>
   <si>
     <t>I-4</t>
@@ -990,7 +990,7 @@
     <t>Draft a block from a screenshot or photo of the client's existing section, plus an optional description</t>
   </si>
   <si>
-    <t>Prototype fakes this — tab 8</t>
+    <t>Prototype fakes this, tab 8</t>
   </si>
   <si>
     <t>FR-M4-7</t>
@@ -1071,7 +1071,7 @@
     <t>Override a placed block's layout and appearance for this document (blocks[i].style)</t>
   </si>
   <si>
-    <t>BLOCKING — see OQ-2</t>
+    <t>BLOCKING, see OQ-2</t>
   </si>
   <si>
     <t>Currently live in the prototype</t>
@@ -1302,7 +1302,7 @@
     <t>BR-12</t>
   </si>
   <si>
-    <t>The admin workspace carries no per-field permissions. Who may edit what is decided in the client editor — owner decides, estimator obeys.</t>
+    <t>The admin workspace carries no per-field permissions. Who may edit what is decided in the client editor: owner decides, estimator obeys.</t>
   </si>
   <si>
     <t>Keeps the admin builders simple; one place owns permissions</t>
@@ -1413,7 +1413,7 @@
     <t>Real extraction from PDF / DOCX</t>
   </si>
   <si>
-    <t>9. Data model — the contract for the build</t>
+    <t>9. Data model, the contract for the build</t>
   </si>
   <si>
     <t>As modelled in the prototype. Field names are the contract the client-side editor must be specified against.</t>
@@ -1557,7 +1557,7 @@
     <t>OQ-1</t>
   </si>
   <si>
-    <t>What does onboarding one client actually cost — admin hours, and lead time to a fillable template? Who performs it?</t>
+    <t>What does onboarding one client actually cost: admin hours, and lead time to a fillable template? Who performs it?</t>
   </si>
   <si>
     <t>Tom</t>
@@ -1593,7 +1593,7 @@
     <t>OQ-3</t>
   </si>
   <si>
-    <t>Brand is a log, not versions — but an issued tender pins a snapshot. Is a real version record required for v1?</t>
+    <t>Brand is a log, not versions, but an issued tender pins a snapshot. Is a real version record required for v1?</t>
   </si>
   <si>
     <t>Shivam</t>
@@ -1764,7 +1764,7 @@
     <t>Onboarding cost makes admin-built uneconomic at scale</t>
   </si>
   <si>
-    <t>OQ-1 — measure before committing to the model</t>
+    <t>OQ-1: measure before committing to the model</t>
   </si>
   <si>
     <t>R-2</t>
@@ -1773,7 +1773,7 @@
     <t>Styling ownership left open; override plumbing built then deleted</t>
   </si>
   <si>
-    <t>OQ-2 — decide before the client-side sprint</t>
+    <t>OQ-2: decide before the client-side sprint</t>
   </si>
   <si>
     <t>R-3</t>

</xml_diff>